<commit_message>
feat(review): nhãn model cho 256 dòng T6 theo hướng dẫn 2.0, phiếu audit T6
- 256 nhãn claude-opus-5-5 cho 128 lineage T6 ranh_gioi ngoài D4 và pilot;
  93 nhãn bắt buộc audit trong data/review/audit_T6.xlsx (W1-13).
- Hướng dẫn 2.0 làm rõ 14/10: câu ghép có/không + nội dung; cơ quan kế
  thừa và địa danh đổi tên do sáp nhập trong quy trình chuyển chỗ.
- crosscheck_evidence.py nhận --ids, --out cho dòng bất kỳ của release.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/review/crosscheck_A.xlsx
+++ b/data/review/crosscheck_A.xlsx
@@ -746,7 +746,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>T6   Hết hiệu lực một phần ở cấp Khoản/Điểm. Cột đáp án ghi "(không có đáp án: ...)". Câu hỏi không được là dạng có/không. Nếu nội dung đã CHUYỂN CHỖ (đạt đủ 7 yếu tố, hướng dẫn §3) thì đáp án rỗng là sai: khong_dat, gold_wrong, ghi chỗ mới vào note. Không chắc thì vẫn dat (nếu không có lỗi khác) và ghi "unclear" vào note.</t>
+          <t>T6   Hết hiệu lực một phần ở cấp Khoản/Điểm. Cột đáp án ghi "(không có đáp án: ...)". Câu CHỈ hỏi có/không là group_mismatch; câu ghép có thêm vế hỏi nội dung ("... có áp dụng không, và quy định cụ thể thế nào?") thì chấm theo vế nội dung. Nếu nội dung đã CHUYỂN CHỖ (đạt đủ 7 yếu tố, hướng dẫn §3) thì đáp án rỗng là sai: khong_dat, gold_wrong, ghi chỗ mới vào note. Sáp nhập: cơ quan kế thừa (Bộ GTVT vào Bộ Xây dựng) đạt yếu tố 6; địa danh chỉ đổi tên do sáp nhập tỉnh/xã, phạm vi và ranh giới giữ nguyên (Bến Tre thành Vĩnh Long) đạt yếu tố 2. Không chắc thì vẫn dat (nếu không có lỗi khác) và ghi "unclear" vào note.</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi không làm được việc của nhóm. T2 không chạm chỗ thay đổi (hai mốc trả lời như nhau); T3 chỉ chạm một lần sửa; T6 hỏi kiểu có/không; T5 hỏi vào phần không đổi.</t>
+          <t>Câu hỏi không làm được việc của nhóm. T2 không chạm chỗ thay đổi (hai mốc trả lời như nhau); T3 chỉ chạm một lần sửa; T6 CHỈ hỏi có/không (câu ghép có thêm vế hỏi nội dung thì không tính); T5 hỏi vào phần không đổi.</t>
         </is>
       </c>
     </row>

</xml_diff>